<commit_message>
working tender; updating vaccine allocation
</commit_message>
<xml_diff>
--- a/Heuristic/data/Starting_point.xlsx
+++ b/Heuristic/data/Starting_point.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28025"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Vaccine_Tender/Heuristic/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="98" documentId="13_ncr:1_{E4667220-B6D3-44CA-BB2C-7EE709A98D96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{98C0F0CD-4487-4EAF-8770-9D482198FB14}"/>
+  <xr:revisionPtr revIDLastSave="99" documentId="13_ncr:1_{E4667220-B6D3-44CA-BB2C-7EE709A98D96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C259262-6517-4957-BCCE-4EE5F2B0DB0F}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="F_start" sheetId="2" r:id="rId1"/>
@@ -263,7 +263,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -289,6 +289,7 @@
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -715,13 +716,13 @@
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="14" t="s">
+      <c r="A13" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="14">
-        <v>1</v>
-      </c>
-      <c r="C13" s="14">
+      <c r="B13" s="15">
+        <v>1</v>
+      </c>
+      <c r="C13" s="15">
         <v>3</v>
       </c>
     </row>

</xml_diff>